<commit_message>
feat(liquidacion): formatos Word y Excel rediseñados en una sola pagina
- Word: encabezado con empresa y periodo, ficha del trabajador en cuadricula,
  haberes y descuentos lado a lado, bases de calculo, liquido a pagar
  destacado, forma de pago y firmas. Cabe en una hoja carta (antes, dos).
- Excel: mismo diseño con las formulas de AFP, salud, cesantia, impuesto
  unico y liquido. Verificado con los tres casos de prueba (sueldo minimo
  $452.917, $1.500.000 Habitat y $4.000.000 Isapre con tope).
- Pagina: descripciones actualizadas y ?v=2 en los enlaces para no servir
  la version en cache.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLXjYYN7g49YRmmeLkdTX3
</commit_message>
<xml_diff>
--- a/descargas/formato-liquidacion-de-sueldo.xlsx
+++ b/descargas/formato-liquidacion-de-sueldo.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parámetros" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Liquidación'!$A$1:$B$56</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Liquidación'!$A$1:$E$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0;-&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,30 +40,80 @@
       <b val="1"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001E293B"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0000382E"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="0064748B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001E293B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0000382E"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001E293B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001E293B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFB703"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00475569"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="0000382E"/>
-    </font>
-    <font>
-      <color rgb="00475569"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00475569"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00D9E6E3"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="0064748B"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="0064748B"/>
+      <sz val="7"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -72,7 +122,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0000382E"/>
+        <fgColor rgb="00FFFBEA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F4"/>
       </patternFill>
     </fill>
     <fill>
@@ -82,21 +137,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFBEA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFB703"/>
+        <fgColor rgb="0000382E"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -105,56 +150,111 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="00CBD5E1"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
+      <bottom style="thick">
+        <color rgb="0000382E"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D7DEE4"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="0000382E"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="medium">
+        <color rgb="0000382E"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="0000382E"/>
+      </bottom>
+    </border>
+    <border>
       <top style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="001E293B"/>
       </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E1"/>
-      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -525,453 +625,546 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B56"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="2.5" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>[Razón social de la empresa]</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
           <t>LIQUIDACIÓN DE SUELDO</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Las celdas amarillas se llenan a mano. El resto se calcula solo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Datos del empleador</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Razón social</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>RUT empleador</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Dirección</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Datos del trabajador</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Nombre completo</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RUT: </t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Período</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Septiembre 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dirección: </t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="6" customHeight="1">
+      <c r="A4" s="6" t="n"/>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+    </row>
+    <row r="6" ht="17" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Nombre del trabajador</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>RUT trabajador</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr"/>
+    </row>
+    <row r="7" ht="17" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Cargo</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Fecha de ingreso</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Tipo de contrato</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Indefinido</t>
         </is>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>AFP</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Modelo</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Sistema de salud</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Fonasa</t>
         </is>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Plan Isapre pactado en pesos (si aplica)</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Período (mes y año)</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Plan Isapre en pesos (si aplica)</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Días trabajados</t>
         </is>
       </c>
-      <c r="B19" s="5" t="n">
+      <c r="B10" s="8" t="n">
         <v>30</v>
       </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Haberes imponibles</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Jornada semanal</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>42 horas</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>HABERES IMPONIBLES</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>MONTO</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>DESCUENTOS LEGALES</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>MONTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="17" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Sueldo base</t>
         </is>
       </c>
-      <c r="B22" s="6" t="n">
+      <c r="B13" s="9" t="n">
         <v>553553</v>
       </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>AFP (10% + comisión)</t>
+        </is>
+      </c>
+      <c r="E13" s="13">
+        <f>ROUND(MIN(B19,'Parámetros'!$B$5*'Parámetros'!$B$4)*VLOOKUP(E8,'Parámetros'!$A$10:$B$16,2,FALSE),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>Gratificación</t>
         </is>
       </c>
-      <c r="B23" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="B14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>Salud (7% o plan Isapre)</t>
+        </is>
+      </c>
+      <c r="E14" s="13">
+        <f>IF(B9="Isapre",MAX(ROUND(MIN(B19,'Parámetros'!$B$5*'Parámetros'!$B$4)*0.07,0),E9),ROUND(MIN(B19,'Parámetros'!$B$5*'Parámetros'!$B$4)*0.07,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>Horas extra</t>
         </is>
       </c>
-      <c r="B24" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>Comisiones y bonos</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="B15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Seguro de cesantía (0,6%)</t>
+        </is>
+      </c>
+      <c r="E15" s="13">
+        <f>IF(B8="Indefinido",ROUND(MIN(B19,'Parámetros'!$B$6*'Parámetros'!$B$4)*0.006,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="17" customHeight="1">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Comisiones</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Impuesto único</t>
+        </is>
+      </c>
+      <c r="E16" s="13">
+        <f>MAX(0,ROUND((B19-E13-MIN(E14,ROUND(MIN(B19,'Parámetros'!$B$5*'Parámetros'!$B$4)*0.07,0))-E15)*LOOKUP((B19-E13-MIN(E14,ROUND(MIN(B19,'Parámetros'!$B$5*'Parámetros'!$B$4)*0.07,0))-E15)/'Parámetros'!$B$3,'Parámetros'!$A$19:$A$26,'Parámetros'!$B$19:$B$26)-LOOKUP((B19-E13-MIN(E14,ROUND(MIN(B19,'Parámetros'!$B$5*'Parámetros'!$B$4)*0.07,0))-E15)/'Parámetros'!$B$3,'Parámetros'!$A$19:$A$26,'Parámetros'!$C$19:$C$26)*'Parámetros'!$B$3,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="17" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Bonos</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>Total descuentos legales</t>
+        </is>
+      </c>
+      <c r="E17" s="15">
+        <f>SUM(E13:E16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="17" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Semana corrida</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>OTROS DESCUENTOS</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>MONTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="17" customHeight="1">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>Total imponible</t>
         </is>
       </c>
-      <c r="B26" s="8">
-        <f>SUM(B22:B25)</f>
+      <c r="B19" s="15">
+        <f>SUM(B13:B18)</f>
         <v/>
       </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>Haberes no imponibles</t>
-        </is>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>Anticipo de sueldo</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" ht="17" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>HABERES NO IMPONIBLES</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>MONTO</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Cuota sindical</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" ht="17" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>Colación</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>Préstamo caja de compensación</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" ht="17" customHeight="1">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>Movilización</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Otros descuentos autorizados</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" ht="17" customHeight="1">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>Viáticos</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>Total otros descuentos</t>
+        </is>
+      </c>
+      <c r="E23" s="15">
+        <f>SUM(E19:E22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="17" customHeight="1">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>Asignación familiar</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" ht="17" customHeight="1">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>Total no imponible</t>
+        </is>
+      </c>
+      <c r="B25" s="15">
+        <f>SUM(B21:B24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="17" customHeight="1"/>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>TOTAL HABERES</t>
+        </is>
+      </c>
+      <c r="B27" s="17">
+        <f>B19+B25</f>
+        <v/>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>TOTAL DESCUENTOS</t>
+        </is>
+      </c>
+      <c r="E27" s="17">
+        <f>E17+E23</f>
+        <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Colación</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="n">
-        <v>0</v>
-      </c>
+      <c r="A29" s="18" t="inlineStr">
+        <is>
+          <t>BASES DE CÁLCULO</t>
+        </is>
+      </c>
+      <c r="D29" s="19" t="inlineStr">
+        <is>
+          <t>LÍQUIDO A PAGAR</t>
+        </is>
+      </c>
+      <c r="E29" s="20" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>Movilización</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="n">
-        <v>0</v>
-      </c>
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>Base imponible AFP y salud</t>
+        </is>
+      </c>
+      <c r="B30" s="13">
+        <f>MIN(B19,'Parámetros'!$B$5*'Parámetros'!$B$4)</f>
+        <v/>
+      </c>
+      <c r="D30" s="21">
+        <f>B27-E27</f>
+        <v/>
+      </c>
+      <c r="E30" s="20" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>Viáticos</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="n">
-        <v>0</v>
-      </c>
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>Base seguro de cesantía</t>
+        </is>
+      </c>
+      <c r="B31" s="13">
+        <f>IF(B8="Indefinido",MIN(B19,'Parámetros'!$B$6*'Parámetros'!$B$4),0)</f>
+        <v/>
+      </c>
+      <c r="D31" s="20" t="n"/>
+      <c r="E31" s="20" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>Total no imponible</t>
-        </is>
-      </c>
-      <c r="B32" s="8">
-        <f>SUM(B29:B31)</f>
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>Base tributable (impuesto único)</t>
+        </is>
+      </c>
+      <c r="B32" s="13">
+        <f>(B19-E13-MIN(E14,ROUND(MIN(B19,'Parámetros'!$B$5*'Parámetros'!$B$4)*0.07,0))-E15)</f>
         <v/>
       </c>
+      <c r="D32" s="20" t="n"/>
+      <c r="E32" s="20" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="9" t="inlineStr">
-        <is>
-          <t>TOTAL HABERES</t>
-        </is>
-      </c>
-      <c r="B33" s="10">
-        <f>B26+B32</f>
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>Valor UTM</t>
+        </is>
+      </c>
+      <c r="B33" s="13">
+        <f>'Parámetros'!$B$3</f>
         <v/>
       </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>Descuentos legales</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>AFP (10% + comisión)</t>
-        </is>
-      </c>
-      <c r="B36" s="11">
-        <f>ROUND(MIN(B26,'Parámetros'!$B$5*'Parámetros'!$B$4)*VLOOKUP(B15,'Parámetros'!$A$10:$B$16,2,FALSE),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>Salud (7% Fonasa o plan Isapre)</t>
-        </is>
-      </c>
-      <c r="B37" s="11">
-        <f>IF(B16="Isapre",MAX(ROUND(MIN(B26,'Parámetros'!$B$5*'Parámetros'!$B$4)*0.07,0),B17),ROUND(MIN(B26,'Parámetros'!$B$5*'Parámetros'!$B$4)*0.07,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>Seguro de cesantía (0,6% si es indefinido)</t>
-        </is>
-      </c>
-      <c r="B38" s="11">
-        <f>IF(B14="Indefinido",ROUND(MIN(B26,'Parámetros'!$B$6*'Parámetros'!$B$4)*0.006,0),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>Renta tributable (base del impuesto)</t>
-        </is>
-      </c>
-      <c r="B39" s="11">
-        <f>B26-B36-MIN(B37,ROUND(MIN(B26,'Parámetros'!$B$5*'Parámetros'!$B$4)*0.07,0))-B38</f>
-        <v/>
+      <c r="D33" s="22" t="inlineStr">
+        <is>
+          <t>Son: ____________________________ pesos</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="26" customHeight="1">
+      <c r="A36" s="23" t="inlineStr">
+        <is>
+          <t>Certifico que he recibido de mi empleador, a mi entera satisfacción, el líquido a pagar indicado en esta liquidación y que no tengo cargo ni cobro alguno que hacer por los conceptos que comprende.</t>
+        </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>Impuesto único de segunda categoría</t>
-        </is>
-      </c>
-      <c r="B40" s="11">
-        <f>MAX(0,ROUND(B39*LOOKUP(B39/'Parámetros'!$B$3,'Parámetros'!$A$19:$A$26,'Parámetros'!$B$19:$B$26)-LOOKUP(B39/'Parámetros'!$B$3,'Parámetros'!$A$19:$A$26,'Parámetros'!$C$19:$C$26)*'Parámetros'!$B$3,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>Otros descuentos</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>Anticipos</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>Otros descuentos autorizados</t>
-        </is>
-      </c>
-      <c r="B44" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="9" t="inlineStr">
-        <is>
-          <t>TOTAL DESCUENTOS</t>
-        </is>
-      </c>
-      <c r="B45" s="10">
-        <f>B36+B37+B38+B40+B43+B44</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="12" t="inlineStr">
-        <is>
-          <t>ALCANCE LÍQUIDO A PAGAR</t>
-        </is>
-      </c>
-      <c r="B47" s="13">
-        <f>B33-B45</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" ht="30" customHeight="1">
-      <c r="A50" s="14" t="inlineStr">
-        <is>
-          <t>Certifico que he recibido de mi empleador, a mi entera satisfacción, el alcance líquido de la presente liquidación.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>______________________________</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>______________________</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A40" s="24" t="inlineStr">
+        <is>
+          <t>Firma y timbre del empleador</t>
+        </is>
+      </c>
+      <c r="B40" s="25" t="n"/>
+      <c r="D40" s="24" t="inlineStr">
         <is>
           <t>Firma del trabajador</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Fecha</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="15" t="inlineStr">
-        <is>
-          <t>Formato gratuito de calculolaboral.cl/liquidacion-de-sueldo. Es un modelo de referencia; revisa los valores con tu contrato.</t>
+      <c r="E40" s="25" t="n"/>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="26" t="inlineStr">
+        <is>
+          <t>Las celdas amarillas se llenan a mano; el resto se calcula solo. Formato gratuito de calculolaboral.cl/liquidacion-de-sueldo. Es un modelo de referencia; revisa los valores con tu contrato.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A50:B50"/>
-    <mergeCell ref="A56:B56"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A35:B35"/>
+  <mergeCells count="8">
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D30:E32"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation sqref="B14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Indefinido,Plazo fijo"</formula1>
     </dataValidation>
-    <dataValidation sqref="B15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>='Parámetros'!$A$10:$A$16</formula1>
     </dataValidation>
-    <dataValidation sqref="B16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Fonasa,Isapre"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup fitToWidth="1"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -979,7 +1172,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -990,7 +1183,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>Parámetros 2026 (actualízalos cuando cambien)</t>
         </is>
@@ -1002,7 +1195,7 @@
           <t>UTM del mes</t>
         </is>
       </c>
-      <c r="B3" s="17" t="n">
+      <c r="B3" s="28" t="n">
         <v>71721</v>
       </c>
     </row>
@@ -1012,7 +1205,7 @@
           <t>UF del último día del mes</t>
         </is>
       </c>
-      <c r="B4" s="17" t="n">
+      <c r="B4" s="28" t="n">
         <v>40975.41</v>
       </c>
     </row>
@@ -1042,17 +1235,17 @@
           <t>Ingreso mínimo mensual</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n">
+      <c r="B7" s="28" t="n">
         <v>553553</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>AFP</t>
         </is>
       </c>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" s="29" t="inlineStr">
         <is>
           <t>Tasa total (10% + comisión)</t>
         </is>
@@ -1064,7 +1257,7 @@
           <t>Modelo</t>
         </is>
       </c>
-      <c r="B10" s="19" t="n">
+      <c r="B10" s="30" t="n">
         <v>0.1058</v>
       </c>
     </row>
@@ -1074,7 +1267,7 @@
           <t>Uno</t>
         </is>
       </c>
-      <c r="B11" s="19" t="n">
+      <c r="B11" s="30" t="n">
         <v>0.1069</v>
       </c>
     </row>
@@ -1084,7 +1277,7 @@
           <t>PlanVital</t>
         </is>
       </c>
-      <c r="B12" s="19" t="n">
+      <c r="B12" s="30" t="n">
         <v>0.1116</v>
       </c>
     </row>
@@ -1094,7 +1287,7 @@
           <t>Habitat</t>
         </is>
       </c>
-      <c r="B13" s="19" t="n">
+      <c r="B13" s="30" t="n">
         <v>0.1127</v>
       </c>
     </row>
@@ -1104,7 +1297,7 @@
           <t>Capital</t>
         </is>
       </c>
-      <c r="B14" s="19" t="n">
+      <c r="B14" s="30" t="n">
         <v>0.1144</v>
       </c>
     </row>
@@ -1114,7 +1307,7 @@
           <t>Cuprum</t>
         </is>
       </c>
-      <c r="B15" s="19" t="n">
+      <c r="B15" s="30" t="n">
         <v>0.1144</v>
       </c>
     </row>
@@ -1124,22 +1317,22 @@
           <t>Provida</t>
         </is>
       </c>
-      <c r="B16" s="19" t="n">
+      <c r="B16" s="30" t="n">
         <v>0.1145</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="18" t="inlineStr">
+      <c r="A18" s="29" t="inlineStr">
         <is>
           <t>Impuesto único: desde (UTM)</t>
         </is>
       </c>
-      <c r="B18" s="18" t="inlineStr">
+      <c r="B18" s="29" t="inlineStr">
         <is>
           <t>Factor</t>
         </is>
       </c>
-      <c r="C18" s="18" t="inlineStr">
+      <c r="C18" s="29" t="inlineStr">
         <is>
           <t>Rebaja (UTM)</t>
         </is>
@@ -1149,7 +1342,7 @@
       <c r="A19" t="n">
         <v>0</v>
       </c>
-      <c r="B19" s="20" t="n">
+      <c r="B19" s="31" t="n">
         <v>0</v>
       </c>
       <c r="C19" t="n">
@@ -1160,7 +1353,7 @@
       <c r="A20" t="n">
         <v>13.5</v>
       </c>
-      <c r="B20" s="20" t="n">
+      <c r="B20" s="31" t="n">
         <v>0.04</v>
       </c>
       <c r="C20" t="n">
@@ -1171,7 +1364,7 @@
       <c r="A21" t="n">
         <v>30</v>
       </c>
-      <c r="B21" s="20" t="n">
+      <c r="B21" s="31" t="n">
         <v>0.08</v>
       </c>
       <c r="C21" t="n">
@@ -1182,7 +1375,7 @@
       <c r="A22" t="n">
         <v>50</v>
       </c>
-      <c r="B22" s="20" t="n">
+      <c r="B22" s="31" t="n">
         <v>0.135</v>
       </c>
       <c r="C22" t="n">
@@ -1193,7 +1386,7 @@
       <c r="A23" t="n">
         <v>70</v>
       </c>
-      <c r="B23" s="20" t="n">
+      <c r="B23" s="31" t="n">
         <v>0.23</v>
       </c>
       <c r="C23" t="n">
@@ -1204,7 +1397,7 @@
       <c r="A24" t="n">
         <v>90</v>
       </c>
-      <c r="B24" s="20" t="n">
+      <c r="B24" s="31" t="n">
         <v>0.304</v>
       </c>
       <c r="C24" t="n">
@@ -1215,7 +1408,7 @@
       <c r="A25" t="n">
         <v>120</v>
       </c>
-      <c r="B25" s="20" t="n">
+      <c r="B25" s="31" t="n">
         <v>0.35</v>
       </c>
       <c r="C25" t="n">
@@ -1226,7 +1419,7 @@
       <c r="A26" t="n">
         <v>310</v>
       </c>
-      <c r="B26" s="20" t="n">
+      <c r="B26" s="31" t="n">
         <v>0.4</v>
       </c>
       <c r="C26" t="n">
@@ -1235,5 +1428,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(liquidacion): recuadro del liquido a pagar apto para imprimir en blanco y negro
El fondo verde oscuro gastaba tinta y en blanco y negro quedaba como un bloque
gris. Ahora el recuadro (Word y Excel) tiene fondo casi blanco, borde grueso
oscuro y el monto en negro.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLXjYYN7g49YRmmeLkdTX3
</commit_message>
<xml_diff>
--- a/descargas/formato-liquidacion-de-sueldo.xlsx
+++ b/descargas/formato-liquidacion-de-sueldo.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0;-&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -88,18 +88,12 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFB703"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="00000000"/>
       <sz val="22"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00D9E6E3"/>
+      <color rgb="001E293B"/>
       <sz val="8"/>
     </font>
     <font>
@@ -137,11 +131,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0000382E"/>
+        <fgColor rgb="00F4F6F5"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -173,6 +167,48 @@
       </bottom>
     </border>
     <border>
+      <left style="thick">
+        <color rgb="001E293B"/>
+      </left>
+      <top style="thick">
+        <color rgb="001E293B"/>
+      </top>
+    </border>
+    <border>
+      <right style="thick">
+        <color rgb="001E293B"/>
+      </right>
+      <top style="thick">
+        <color rgb="001E293B"/>
+      </top>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="001E293B"/>
+      </left>
+    </border>
+    <border>
+      <right style="thick">
+        <color rgb="001E293B"/>
+      </right>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="001E293B"/>
+      </left>
+      <bottom style="thick">
+        <color rgb="001E293B"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="thick">
+        <color rgb="001E293B"/>
+      </right>
+      <bottom style="thick">
+        <color rgb="001E293B"/>
+      </bottom>
+    </border>
+    <border>
       <top style="thin">
         <color rgb="001E293B"/>
       </top>
@@ -181,7 +217,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -235,24 +271,27 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1068,7 +1107,7 @@
         <f>B27-E27</f>
         <v/>
       </c>
-      <c r="E30" s="20" t="n"/>
+      <c r="E30" s="22" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
@@ -1080,8 +1119,8 @@
         <f>IF(B8="Indefinido",MIN(B19,'Parámetros'!$B$6*'Parámetros'!$B$4),0)</f>
         <v/>
       </c>
-      <c r="D31" s="20" t="n"/>
-      <c r="E31" s="20" t="n"/>
+      <c r="D31" s="23" t="n"/>
+      <c r="E31" s="22" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="12" t="inlineStr">
@@ -1093,8 +1132,8 @@
         <f>(B19-E13-MIN(E14,ROUND(MIN(B19,'Parámetros'!$B$5*'Parámetros'!$B$4)*0.07,0))-E15)</f>
         <v/>
       </c>
-      <c r="D32" s="20" t="n"/>
-      <c r="E32" s="20" t="n"/>
+      <c r="D32" s="23" t="n"/>
+      <c r="E32" s="22" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
@@ -1106,35 +1145,36 @@
         <f>'Parámetros'!$B$3</f>
         <v/>
       </c>
-      <c r="D33" s="22" t="inlineStr">
+      <c r="D33" s="24" t="inlineStr">
         <is>
           <t>Son: ____________________________ pesos</t>
         </is>
       </c>
+      <c r="E33" s="25" t="n"/>
     </row>
     <row r="36" ht="26" customHeight="1">
-      <c r="A36" s="23" t="inlineStr">
+      <c r="A36" s="26" t="inlineStr">
         <is>
           <t>Certifico que he recibido de mi empleador, a mi entera satisfacción, el líquido a pagar indicado en esta liquidación y que no tengo cargo ni cobro alguno que hacer por los conceptos que comprende.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="24" t="inlineStr">
+      <c r="A40" s="27" t="inlineStr">
         <is>
           <t>Firma y timbre del empleador</t>
         </is>
       </c>
-      <c r="B40" s="25" t="n"/>
-      <c r="D40" s="24" t="inlineStr">
+      <c r="B40" s="28" t="n"/>
+      <c r="D40" s="27" t="inlineStr">
         <is>
           <t>Firma del trabajador</t>
         </is>
       </c>
-      <c r="E40" s="25" t="n"/>
+      <c r="E40" s="28" t="n"/>
     </row>
     <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="26" t="inlineStr">
+      <c r="A42" s="29" t="inlineStr">
         <is>
           <t>Las celdas amarillas se llenan a mano; el resto se calcula solo. Formato gratuito de calculolaboral.cl/liquidacion-de-sueldo. Es un modelo de referencia; revisa los valores con tu contrato.</t>
         </is>
@@ -1183,7 +1223,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="27" t="inlineStr">
+      <c r="A1" s="30" t="inlineStr">
         <is>
           <t>Parámetros 2026 (actualízalos cuando cambien)</t>
         </is>
@@ -1195,7 +1235,7 @@
           <t>UTM del mes</t>
         </is>
       </c>
-      <c r="B3" s="28" t="n">
+      <c r="B3" s="31" t="n">
         <v>71721</v>
       </c>
     </row>
@@ -1205,7 +1245,7 @@
           <t>UF del último día del mes</t>
         </is>
       </c>
-      <c r="B4" s="28" t="n">
+      <c r="B4" s="31" t="n">
         <v>40975.41</v>
       </c>
     </row>
@@ -1235,17 +1275,17 @@
           <t>Ingreso mínimo mensual</t>
         </is>
       </c>
-      <c r="B7" s="28" t="n">
+      <c r="B7" s="31" t="n">
         <v>553553</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="29" t="inlineStr">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>AFP</t>
         </is>
       </c>
-      <c r="B9" s="29" t="inlineStr">
+      <c r="B9" s="32" t="inlineStr">
         <is>
           <t>Tasa total (10% + comisión)</t>
         </is>
@@ -1257,7 +1297,7 @@
           <t>Modelo</t>
         </is>
       </c>
-      <c r="B10" s="30" t="n">
+      <c r="B10" s="33" t="n">
         <v>0.1058</v>
       </c>
     </row>
@@ -1267,7 +1307,7 @@
           <t>Uno</t>
         </is>
       </c>
-      <c r="B11" s="30" t="n">
+      <c r="B11" s="33" t="n">
         <v>0.1069</v>
       </c>
     </row>
@@ -1277,7 +1317,7 @@
           <t>PlanVital</t>
         </is>
       </c>
-      <c r="B12" s="30" t="n">
+      <c r="B12" s="33" t="n">
         <v>0.1116</v>
       </c>
     </row>
@@ -1287,7 +1327,7 @@
           <t>Habitat</t>
         </is>
       </c>
-      <c r="B13" s="30" t="n">
+      <c r="B13" s="33" t="n">
         <v>0.1127</v>
       </c>
     </row>
@@ -1297,7 +1337,7 @@
           <t>Capital</t>
         </is>
       </c>
-      <c r="B14" s="30" t="n">
+      <c r="B14" s="33" t="n">
         <v>0.1144</v>
       </c>
     </row>
@@ -1307,7 +1347,7 @@
           <t>Cuprum</t>
         </is>
       </c>
-      <c r="B15" s="30" t="n">
+      <c r="B15" s="33" t="n">
         <v>0.1144</v>
       </c>
     </row>
@@ -1317,22 +1357,22 @@
           <t>Provida</t>
         </is>
       </c>
-      <c r="B16" s="30" t="n">
+      <c r="B16" s="33" t="n">
         <v>0.1145</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="29" t="inlineStr">
+      <c r="A18" s="32" t="inlineStr">
         <is>
           <t>Impuesto único: desde (UTM)</t>
         </is>
       </c>
-      <c r="B18" s="29" t="inlineStr">
+      <c r="B18" s="32" t="inlineStr">
         <is>
           <t>Factor</t>
         </is>
       </c>
-      <c r="C18" s="29" t="inlineStr">
+      <c r="C18" s="32" t="inlineStr">
         <is>
           <t>Rebaja (UTM)</t>
         </is>
@@ -1342,7 +1382,7 @@
       <c r="A19" t="n">
         <v>0</v>
       </c>
-      <c r="B19" s="31" t="n">
+      <c r="B19" s="34" t="n">
         <v>0</v>
       </c>
       <c r="C19" t="n">
@@ -1353,7 +1393,7 @@
       <c r="A20" t="n">
         <v>13.5</v>
       </c>
-      <c r="B20" s="31" t="n">
+      <c r="B20" s="34" t="n">
         <v>0.04</v>
       </c>
       <c r="C20" t="n">
@@ -1364,7 +1404,7 @@
       <c r="A21" t="n">
         <v>30</v>
       </c>
-      <c r="B21" s="31" t="n">
+      <c r="B21" s="34" t="n">
         <v>0.08</v>
       </c>
       <c r="C21" t="n">
@@ -1375,7 +1415,7 @@
       <c r="A22" t="n">
         <v>50</v>
       </c>
-      <c r="B22" s="31" t="n">
+      <c r="B22" s="34" t="n">
         <v>0.135</v>
       </c>
       <c r="C22" t="n">
@@ -1386,7 +1426,7 @@
       <c r="A23" t="n">
         <v>70</v>
       </c>
-      <c r="B23" s="31" t="n">
+      <c r="B23" s="34" t="n">
         <v>0.23</v>
       </c>
       <c r="C23" t="n">
@@ -1397,7 +1437,7 @@
       <c r="A24" t="n">
         <v>90</v>
       </c>
-      <c r="B24" s="31" t="n">
+      <c r="B24" s="34" t="n">
         <v>0.304</v>
       </c>
       <c r="C24" t="n">
@@ -1408,7 +1448,7 @@
       <c r="A25" t="n">
         <v>120</v>
       </c>
-      <c r="B25" s="31" t="n">
+      <c r="B25" s="34" t="n">
         <v>0.35</v>
       </c>
       <c r="C25" t="n">
@@ -1419,7 +1459,7 @@
       <c r="A26" t="n">
         <v>310</v>
       </c>
-      <c r="B26" s="31" t="n">
+      <c r="B26" s="34" t="n">
         <v>0.4</v>
       </c>
       <c r="C26" t="n">

</xml_diff>